<commit_message>
Update columns_by_dataset and the raw metadata exploration notebook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/metadata/columns_by_dataset.xlsx
+++ b/assets/metadata/columns_by_dataset.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G155"/>
+  <dimension ref="A1:H176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -445,14 +445,11 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>colonna</t>
-        </is>
-      </c>
+      <c r="A1" s="1" t="n"/>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>PASPORT</t>
@@ -475,10 +472,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>UKE_SFB</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>UKLFR</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>WashU</t>
         </is>
@@ -516,6 +518,11 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -549,11 +556,16 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>lesion_side</t>
+          <t>NIHSS</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
@@ -578,11 +590,16 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NIHSS</t>
+          <t>lesion_side</t>
         </is>
       </c>
       <c r="B5" s="3" t="n"/>
@@ -607,6 +624,11 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -636,11 +658,16 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NIHSS_2</t>
+          <t>participant_id_dmp</t>
         </is>
       </c>
       <c r="B7" s="3" t="n"/>
@@ -661,27 +688,37 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NIHSS_4</t>
+          <t>acq_time</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D8" s="3" t="n"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E8" s="3" t="n"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -690,23 +727,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>clinical_date</t>
+          <t>NIHSS_7</t>
         </is>
       </c>
       <c r="B9" s="3" t="n"/>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n"/>
       <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -715,23 +753,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NIHSS_3</t>
+          <t>clinical_date</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D10" s="3" t="n"/>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
       <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -740,7 +779,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NIHSS_8</t>
+          <t>NIHSS_2</t>
         </is>
       </c>
       <c r="B11" s="3" t="n"/>
@@ -751,12 +790,13 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F11" s="3" t="n"/>
       <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -765,7 +805,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NIHSS_9</t>
+          <t>diagnosis_date</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -786,27 +826,29 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>acq_time</t>
+          <t>NIHSS_3</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n"/>
       <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -815,7 +857,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NIHSS_7</t>
+          <t>NIHSS_4</t>
         </is>
       </c>
       <c r="B14" s="3" t="n"/>
@@ -826,12 +868,13 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F14" s="3" t="n"/>
       <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -840,14 +883,10 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>mRS_3m</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>NIHSS_11</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="2" t="inlineStr">
@@ -855,17 +894,22 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NIHSS_11</t>
+          <t>NIHSS_10</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
@@ -876,12 +920,13 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F16" s="3" t="n"/>
       <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -890,10 +935,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NIHSS_10</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n"/>
+          <t>NIHSS_3m</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="2" t="inlineStr">
@@ -906,16 +955,13 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>participant_id_dmp</t>
+          <t>NIHSS_9</t>
         </is>
       </c>
       <c r="B18" s="3" t="n"/>
@@ -926,12 +972,13 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F18" s="3" t="n"/>
       <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -940,7 +987,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NIHSS_1C</t>
+          <t>NIHSS_8</t>
         </is>
       </c>
       <c r="B19" s="3" t="n"/>
@@ -957,14 +1004,23 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NIHSS_1B</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n"/>
+          <t>mRS_3m</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="2" t="inlineStr">
@@ -978,11 +1034,12 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NIHSS_1A</t>
+          <t>NIHSS_5a</t>
         </is>
       </c>
       <c r="B21" s="3" t="n"/>
@@ -999,6 +1056,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1020,53 +1078,56 @@
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Token</t>
+          <t>NIHSS_6b</t>
         </is>
       </c>
       <c r="B23" s="3" t="n"/>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C23" s="3" t="n"/>
       <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="n"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Digit_forw</t>
+          <t>NIHSS_1B</t>
         </is>
       </c>
       <c r="B24" s="3" t="n"/>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C24" s="3" t="n"/>
       <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Digit_back</t>
+          <t>behavioral_date</t>
         </is>
       </c>
       <c r="B25" s="3" t="n"/>
@@ -1077,38 +1138,40 @@
       </c>
       <c r="D25" s="3" t="n"/>
       <c r="E25" s="3" t="n"/>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NIHSS_6a</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
+          <t>mRS_pre_stroke</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D26" s="3" t="n"/>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NIHSS_5a</t>
+          <t>NIHSS_1A</t>
         </is>
       </c>
       <c r="B27" s="3" t="n"/>
@@ -1119,17 +1182,18 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>behavioral_date</t>
+          <t>NIHSS_12m</t>
         </is>
       </c>
       <c r="B28" s="3" t="n"/>
@@ -1140,38 +1204,40 @@
       </c>
       <c r="D28" s="3" t="n"/>
       <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Corsi</t>
+          <t>Digit_forw</t>
         </is>
       </c>
       <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D29" s="3" t="n"/>
       <c r="E29" s="3" t="n"/>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F29" s="3" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
+      <c r="H29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Boston_nam</t>
+          <t>Digit_back</t>
         </is>
       </c>
       <c r="B30" s="3" t="n"/>
@@ -1188,32 +1254,34 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NIHSS_6b</t>
+          <t>NIHSS_6m</t>
         </is>
       </c>
       <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D31" s="3" t="n"/>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>diagnosis_date</t>
+          <t>NIHSS_5b</t>
         </is>
       </c>
       <c r="B32" s="3" t="n"/>
@@ -1224,45 +1292,43 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>mRS_pre_stroke</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>&lt;gene nomenclature&gt;</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
       <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>NIHSS_3m</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>NIHSS_6a</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n"/>
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="3" t="n"/>
       <c r="E34" s="2" t="inlineStr">
@@ -1271,54 +1337,61 @@
         </is>
       </c>
       <c r="F34" s="3" t="n"/>
-      <c r="G34" s="3" t="n"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>NIHSS_6m</t>
+          <t>Corsi</t>
         </is>
       </c>
       <c r="B35" s="3" t="n"/>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C35" s="3" t="n"/>
       <c r="D35" s="3" t="n"/>
       <c r="E35" s="3" t="n"/>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>NIHSS_5b</t>
+          <t>Boston_nam</t>
         </is>
       </c>
       <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D36" s="3" t="n"/>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="n"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OCS_Egocentric_neglect</t>
+          <t>Token</t>
         </is>
       </c>
       <c r="B37" s="3" t="n"/>
@@ -1330,29 +1403,39 @@
       <c r="D37" s="3" t="n"/>
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OCS_Executive_function_mixed</t>
+          <t>NIHSS_1C</t>
         </is>
       </c>
       <c r="B38" s="3" t="n"/>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C38" s="3" t="n"/>
       <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OCS_Executive_function_difference</t>
+          <t>OCS_Orientation</t>
         </is>
       </c>
       <c r="B39" s="3" t="n"/>
@@ -1365,28 +1448,30 @@
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3" t="n"/>
       <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NIHSS_6b_3m</t>
+          <t>OCS_Heart_overrall_accuracy</t>
         </is>
       </c>
       <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D40" s="3" t="n"/>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
       <c r="G40" s="3" t="n"/>
+      <c r="H40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>OCS_Executive_function_circles</t>
+          <t>OCS_Executive_function_tot</t>
         </is>
       </c>
       <c r="B41" s="3" t="n"/>
@@ -1399,11 +1484,12 @@
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="3" t="n"/>
       <c r="G41" s="3" t="n"/>
+      <c r="H41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OCS_Episodic_memory</t>
+          <t>OCS_Number_writing</t>
         </is>
       </c>
       <c r="B42" s="3" t="n"/>
@@ -1416,11 +1502,12 @@
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3" t="n"/>
       <c r="G42" s="3" t="n"/>
+      <c r="H42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OCS_Executive_function_tot</t>
+          <t>OCS_Imitating_gesture_dominant_hand</t>
         </is>
       </c>
       <c r="B43" s="3" t="n"/>
@@ -1433,11 +1520,12 @@
       <c r="E43" s="3" t="n"/>
       <c r="F43" s="3" t="n"/>
       <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OCS_Denomination</t>
+          <t>OCS_Executive_function_squares</t>
         </is>
       </c>
       <c r="B44" s="3" t="n"/>
@@ -1450,11 +1538,12 @@
       <c r="E44" s="3" t="n"/>
       <c r="F44" s="3" t="n"/>
       <c r="G44" s="3" t="n"/>
+      <c r="H44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OCS_Calculation</t>
+          <t>OCS_Denomination</t>
         </is>
       </c>
       <c r="B45" s="3" t="n"/>
@@ -1467,11 +1556,12 @@
       <c r="E45" s="3" t="n"/>
       <c r="F45" s="3" t="n"/>
       <c r="G45" s="3" t="n"/>
+      <c r="H45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OCS_Allocentric_neglect</t>
+          <t>OCS_Executive_function_mixed</t>
         </is>
       </c>
       <c r="B46" s="3" t="n"/>
@@ -1484,11 +1574,12 @@
       <c r="E46" s="3" t="n"/>
       <c r="F46" s="3" t="n"/>
       <c r="G46" s="3" t="n"/>
+      <c r="H46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OCS</t>
+          <t>OCS_Executive_function_difference</t>
         </is>
       </c>
       <c r="B47" s="3" t="n"/>
@@ -1501,79 +1592,84 @@
       <c r="E47" s="3" t="n"/>
       <c r="F47" s="3" t="n"/>
       <c r="G47" s="3" t="n"/>
+      <c r="H47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>NIHSS_at_presentation</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="n"/>
+          <t>OCS_Executive_function_circles</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n"/>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D48" s="3" t="n"/>
       <c r="E48" s="3" t="n"/>
       <c r="F48" s="3" t="n"/>
       <c r="G48" s="3" t="n"/>
+      <c r="H48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NIHSS_7_3m</t>
+          <t>OCS_Episodic_memory</t>
         </is>
       </c>
       <c r="B49" s="3" t="n"/>
-      <c r="C49" s="3" t="n"/>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D49" s="3" t="n"/>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E49" s="3" t="n"/>
       <c r="F49" s="3" t="n"/>
       <c r="G49" s="3" t="n"/>
+      <c r="H49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>NIHSS_9_3m</t>
+          <t>OCS_Egocentric_neglect</t>
         </is>
       </c>
       <c r="B50" s="3" t="n"/>
-      <c r="C50" s="3" t="n"/>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D50" s="3" t="n"/>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E50" s="3" t="n"/>
       <c r="F50" s="3" t="n"/>
       <c r="G50" s="3" t="n"/>
+      <c r="H50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>NIHSS_8_3m</t>
+          <t>OCS_Sentence_reading</t>
         </is>
       </c>
       <c r="B51" s="3" t="n"/>
-      <c r="C51" s="3" t="n"/>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D51" s="3" t="n"/>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E51" s="3" t="n"/>
       <c r="F51" s="3" t="n"/>
       <c r="G51" s="3" t="n"/>
+      <c r="H51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OCS_Executive_function_squares</t>
+          <t>OCS_Calculation</t>
         </is>
       </c>
       <c r="B52" s="3" t="n"/>
@@ -1586,28 +1682,30 @@
       <c r="E52" s="3" t="n"/>
       <c r="F52" s="3" t="n"/>
       <c r="G52" s="3" t="n"/>
+      <c r="H52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>9HPT_L</t>
+          <t>OCS_Allocentric_neglect</t>
         </is>
       </c>
       <c r="B53" s="3" t="n"/>
-      <c r="C53" s="3" t="n"/>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D53" s="3" t="n"/>
       <c r="E53" s="3" t="n"/>
       <c r="F53" s="3" t="n"/>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G53" s="3" t="n"/>
+      <c r="H53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OCS_Heart_overrall_accuracy</t>
+          <t>OCS</t>
         </is>
       </c>
       <c r="B54" s="3" t="n"/>
@@ -1620,45 +1718,48 @@
       <c r="E54" s="3" t="n"/>
       <c r="F54" s="3" t="n"/>
       <c r="G54" s="3" t="n"/>
+      <c r="H54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>gene_nomvenclature</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="n"/>
+          <t>NIHSS_at_presentation</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="C55" s="3" t="n"/>
       <c r="D55" s="3" t="n"/>
       <c r="E55" s="3" t="n"/>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F55" s="3" t="n"/>
       <c r="G55" s="3" t="n"/>
+      <c r="H55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TMT_B</t>
+          <t>NIHSS_9_3m</t>
         </is>
       </c>
       <c r="B56" s="3" t="n"/>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C56" s="3" t="n"/>
       <c r="D56" s="3" t="n"/>
-      <c r="E56" s="3" t="n"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="n"/>
+      <c r="H56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>WBC_Count</t>
+          <t>NIHSS_8_3m</t>
         </is>
       </c>
       <c r="B57" s="3" t="n"/>
@@ -1671,11 +1772,12 @@
       </c>
       <c r="F57" s="3" t="n"/>
       <c r="G57" s="3" t="n"/>
+      <c r="H57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>aPTT</t>
+          <t>NIHSS_7_3m</t>
         </is>
       </c>
       <c r="B58" s="3" t="n"/>
@@ -1688,130 +1790,138 @@
       </c>
       <c r="F58" s="3" t="n"/>
       <c r="G58" s="3" t="n"/>
+      <c r="H58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>acquisition_time</t>
+          <t>OCS_Semantics</t>
         </is>
       </c>
       <c r="B59" s="3" t="n"/>
-      <c r="C59" s="3" t="n"/>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D59" s="3" t="n"/>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E59" s="3" t="n"/>
       <c r="F59" s="3" t="n"/>
       <c r="G59" s="3" t="n"/>
+      <c r="H59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>behavioural_date</t>
+          <t>9HPT_L</t>
         </is>
       </c>
       <c r="B60" s="3" t="n"/>
       <c r="C60" s="3" t="n"/>
       <c r="D60" s="3" t="n"/>
       <c r="E60" s="3" t="n"/>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F60" s="3" t="n"/>
       <c r="G60" s="3" t="n"/>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>codetrt</t>
+          <t>OCS_Verbal_memory</t>
         </is>
       </c>
       <c r="B61" s="3" t="n"/>
-      <c r="C61" s="3" t="n"/>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D61" s="3" t="n"/>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E61" s="3" t="n"/>
       <c r="F61" s="3" t="n"/>
       <c r="G61" s="3" t="n"/>
+      <c r="H61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>lesion_type</t>
+          <t>gripstrength_affected_nonaffected_1m</t>
         </is>
       </c>
       <c r="B62" s="3" t="n"/>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C62" s="3" t="n"/>
       <c r="D62" s="3" t="n"/>
       <c r="E62" s="3" t="n"/>
-      <c r="F62" s="3" t="n"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G62" s="3" t="n"/>
+      <c r="H62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>OCS_Imitating_gesture_dominant_hand</t>
+          <t>gene_nomvenclature</t>
         </is>
       </c>
       <c r="B63" s="3" t="n"/>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C63" s="3" t="n"/>
       <c r="D63" s="3" t="n"/>
       <c r="E63" s="3" t="n"/>
       <c r="F63" s="3" t="n"/>
-      <c r="G63" s="3" t="n"/>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>lesion_volume_ml</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>gripstrength_affected_hand_kg</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="n"/>
       <c r="C64" s="3" t="n"/>
       <c r="D64" s="3" t="n"/>
       <c r="E64" s="3" t="n"/>
-      <c r="F64" s="3" t="n"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G64" s="3" t="n"/>
+      <c r="H64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>mRS</t>
+          <t>gripstrength_affected_hand_kg_12m</t>
         </is>
       </c>
       <c r="B65" s="3" t="n"/>
       <c r="C65" s="3" t="n"/>
       <c r="D65" s="3" t="n"/>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="n"/>
+      <c r="E65" s="3" t="n"/>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G65" s="3" t="n"/>
+      <c r="H65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>mRS_0m</t>
+          <t>gripstrength_affected_hand_kg_1m</t>
         </is>
       </c>
       <c r="B66" s="3" t="n"/>
@@ -1824,11 +1934,12 @@
         </is>
       </c>
       <c r="G66" s="3" t="n"/>
+      <c r="H66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>mRS_6m</t>
+          <t>gripstrength_affected_hand_kg_3m</t>
         </is>
       </c>
       <c r="B67" s="3" t="n"/>
@@ -1841,113 +1952,120 @@
         </is>
       </c>
       <c r="G67" s="3" t="n"/>
+      <c r="H67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>mRS_discharge</t>
+          <t>gripstrength_affected_nonaffected</t>
         </is>
       </c>
       <c r="B68" s="3" t="n"/>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C68" s="3" t="n"/>
       <c r="D68" s="3" t="n"/>
       <c r="E68" s="3" t="n"/>
-      <c r="F68" s="3" t="n"/>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G68" s="3" t="n"/>
+      <c r="H68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>original_id</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>gripstrength_affected_nonaffected_12m</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="n"/>
       <c r="C69" s="3" t="n"/>
       <c r="D69" s="3" t="n"/>
       <c r="E69" s="3" t="n"/>
-      <c r="F69" s="3" t="n"/>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G69" s="3" t="n"/>
+      <c r="H69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TMT_A</t>
+          <t>gripstrength_affected_nonaffected_3m</t>
         </is>
       </c>
       <c r="B70" s="3" t="n"/>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C70" s="3" t="n"/>
       <c r="D70" s="3" t="n"/>
       <c r="E70" s="3" t="n"/>
-      <c r="F70" s="3" t="n"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G70" s="3" t="n"/>
+      <c r="H70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TIA</t>
+          <t>days_since_stroke_1m</t>
         </is>
       </c>
       <c r="B71" s="3" t="n"/>
       <c r="C71" s="3" t="n"/>
       <c r="D71" s="3" t="n"/>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="n"/>
+      <c r="E71" s="3" t="n"/>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G71" s="3" t="n"/>
+      <c r="H71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Statines_drug</t>
+          <t>lesion_type</t>
         </is>
       </c>
       <c r="B72" s="3" t="n"/>
-      <c r="C72" s="3" t="n"/>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D72" s="3" t="n"/>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E72" s="3" t="n"/>
       <c r="F72" s="3" t="n"/>
       <c r="G72" s="3" t="n"/>
+      <c r="H72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Statines</t>
-        </is>
-      </c>
-      <c r="B73" s="3" t="n"/>
+          <t>lesion_volume_ml</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="C73" s="3" t="n"/>
       <c r="D73" s="3" t="n"/>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E73" s="3" t="n"/>
       <c r="F73" s="3" t="n"/>
       <c r="G73" s="3" t="n"/>
+      <c r="H73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Serum_Glucose</t>
+          <t>mRS</t>
         </is>
       </c>
       <c r="B74" s="3" t="n"/>
@@ -1960,45 +2078,48 @@
       </c>
       <c r="F74" s="3" t="n"/>
       <c r="G74" s="3" t="n"/>
+      <c r="H74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>RBC_Count</t>
+          <t>mRS_0m</t>
         </is>
       </c>
       <c r="B75" s="3" t="n"/>
       <c r="C75" s="3" t="n"/>
       <c r="D75" s="3" t="n"/>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E75" s="3" t="n"/>
       <c r="F75" s="3" t="n"/>
-      <c r="G75" s="3" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Prose_memory_imm</t>
+          <t>mRS_6m</t>
         </is>
       </c>
       <c r="B76" s="3" t="n"/>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C76" s="3" t="n"/>
       <c r="D76" s="3" t="n"/>
       <c r="E76" s="3" t="n"/>
       <c r="F76" s="3" t="n"/>
-      <c r="G76" s="3" t="n"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Prose_memory_del</t>
+          <t>mRS_discharge</t>
         </is>
       </c>
       <c r="B77" s="3" t="n"/>
@@ -2011,147 +2132,156 @@
       <c r="E77" s="3" t="n"/>
       <c r="F77" s="3" t="n"/>
       <c r="G77" s="3" t="n"/>
+      <c r="H77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Platelet_aggreg_inhib_drug</t>
-        </is>
-      </c>
-      <c r="B78" s="3" t="n"/>
+          <t>original_id</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="C78" s="3" t="n"/>
       <c r="D78" s="3" t="n"/>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E78" s="3" t="n"/>
       <c r="F78" s="3" t="n"/>
       <c r="G78" s="3" t="n"/>
+      <c r="H78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Platelet_aggreg_inhib</t>
+          <t>days_since_stroke_3m</t>
         </is>
       </c>
       <c r="B79" s="3" t="n"/>
       <c r="C79" s="3" t="n"/>
       <c r="D79" s="3" t="n"/>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F79" s="3" t="n"/>
+      <c r="E79" s="3" t="n"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G79" s="3" t="n"/>
+      <c r="H79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Platelet_Count</t>
+          <t>days_since_stroke_12m</t>
         </is>
       </c>
       <c r="B80" s="3" t="n"/>
       <c r="C80" s="3" t="n"/>
       <c r="D80" s="3" t="n"/>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="n"/>
+      <c r="E80" s="3" t="n"/>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G80" s="3" t="n"/>
+      <c r="H80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>NIHSS_6a_3m</t>
+          <t>OCS_Visual_Field</t>
         </is>
       </c>
       <c r="B81" s="3" t="n"/>
-      <c r="C81" s="3" t="n"/>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D81" s="3" t="n"/>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E81" s="3" t="n"/>
       <c r="F81" s="3" t="n"/>
       <c r="G81" s="3" t="n"/>
+      <c r="H81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>OCS_Verbal_memory</t>
+          <t>Statines_drug</t>
         </is>
       </c>
       <c r="B82" s="3" t="n"/>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C82" s="3" t="n"/>
       <c r="D82" s="3" t="n"/>
-      <c r="E82" s="3" t="n"/>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F82" s="3" t="n"/>
       <c r="G82" s="3" t="n"/>
+      <c r="H82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>OCS_Sentence_reading</t>
+          <t>Platelet_Count</t>
         </is>
       </c>
       <c r="B83" s="3" t="n"/>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C83" s="3" t="n"/>
       <c r="D83" s="3" t="n"/>
-      <c r="E83" s="3" t="n"/>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F83" s="3" t="n"/>
       <c r="G83" s="3" t="n"/>
+      <c r="H83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>OCS_Semantics</t>
+          <t>Platelet_aggreg_inhib</t>
         </is>
       </c>
       <c r="B84" s="3" t="n"/>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C84" s="3" t="n"/>
       <c r="D84" s="3" t="n"/>
-      <c r="E84" s="3" t="n"/>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F84" s="3" t="n"/>
       <c r="G84" s="3" t="n"/>
+      <c r="H84" s="3" t="n"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>OCS_Orientation</t>
+          <t>Platelet_aggreg_inhib_drug</t>
         </is>
       </c>
       <c r="B85" s="3" t="n"/>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C85" s="3" t="n"/>
       <c r="D85" s="3" t="n"/>
-      <c r="E85" s="3" t="n"/>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F85" s="3" t="n"/>
       <c r="G85" s="3" t="n"/>
+      <c r="H85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>OCS_Number_writing</t>
+          <t>Prose_memory_del</t>
         </is>
       </c>
       <c r="B86" s="3" t="n"/>
@@ -2164,11 +2294,12 @@
       <c r="E86" s="3" t="n"/>
       <c r="F86" s="3" t="n"/>
       <c r="G86" s="3" t="n"/>
+      <c r="H86" s="3" t="n"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>OCS_Visual_Field</t>
+          <t>Prose_memory_imm</t>
         </is>
       </c>
       <c r="B87" s="3" t="n"/>
@@ -2181,45 +2312,48 @@
       <c r="E87" s="3" t="n"/>
       <c r="F87" s="3" t="n"/>
       <c r="G87" s="3" t="n"/>
+      <c r="H87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>NIHSS_5A</t>
+          <t>RBC_Count</t>
         </is>
       </c>
       <c r="B88" s="3" t="n"/>
       <c r="C88" s="3" t="n"/>
       <c r="D88" s="3" t="n"/>
-      <c r="E88" s="3" t="n"/>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F88" s="3" t="n"/>
-      <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G88" s="3" t="n"/>
+      <c r="H88" s="3" t="n"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>NIHSS_6B</t>
+          <t>Statines</t>
         </is>
       </c>
       <c r="B89" s="3" t="n"/>
       <c r="C89" s="3" t="n"/>
       <c r="D89" s="3" t="n"/>
-      <c r="E89" s="3" t="n"/>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F89" s="3" t="n"/>
-      <c r="G89" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G89" s="3" t="n"/>
+      <c r="H89" s="3" t="n"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BDI_3m</t>
+          <t>TIA</t>
         </is>
       </c>
       <c r="B90" s="3" t="n"/>
@@ -2232,45 +2366,48 @@
       </c>
       <c r="F90" s="3" t="n"/>
       <c r="G90" s="3" t="n"/>
+      <c r="H90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Gastro_intestinal_bleeding</t>
+          <t>days_since_stroke</t>
         </is>
       </c>
       <c r="B91" s="3" t="n"/>
       <c r="C91" s="3" t="n"/>
       <c r="D91" s="3" t="n"/>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F91" s="3" t="n"/>
+      <c r="E91" s="3" t="n"/>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G91" s="3" t="n"/>
+      <c r="H91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GDS_15</t>
+          <t>TMT_A</t>
         </is>
       </c>
       <c r="B92" s="3" t="n"/>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D92" s="3" t="n"/>
       <c r="E92" s="3" t="n"/>
       <c r="F92" s="3" t="n"/>
-      <c r="G92" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G92" s="3" t="n"/>
+      <c r="H92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Fluency_phonemic</t>
+          <t>TMT_B</t>
         </is>
       </c>
       <c r="B93" s="3" t="n"/>
@@ -2283,11 +2420,12 @@
       <c r="E93" s="3" t="n"/>
       <c r="F93" s="3" t="n"/>
       <c r="G93" s="3" t="n"/>
+      <c r="H93" s="3" t="n"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>FHS_3m</t>
+          <t>WBC_Count</t>
         </is>
       </c>
       <c r="B94" s="3" t="n"/>
@@ -2300,11 +2438,12 @@
       </c>
       <c r="F94" s="3" t="n"/>
       <c r="G94" s="3" t="n"/>
+      <c r="H94" s="3" t="n"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>FHS</t>
+          <t>aPTT</t>
         </is>
       </c>
       <c r="B95" s="3" t="n"/>
@@ -2317,11 +2456,12 @@
       </c>
       <c r="F95" s="3" t="n"/>
       <c r="G95" s="3" t="n"/>
+      <c r="H95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>EQ5D_3m</t>
+          <t>acquisition_time</t>
         </is>
       </c>
       <c r="B96" s="3" t="n"/>
@@ -2334,28 +2474,30 @@
       </c>
       <c r="F96" s="3" t="n"/>
       <c r="G96" s="3" t="n"/>
+      <c r="H96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>EQ5D</t>
+          <t>behavioural_date</t>
         </is>
       </c>
       <c r="B97" s="3" t="n"/>
       <c r="C97" s="3" t="n"/>
       <c r="D97" s="3" t="n"/>
-      <c r="E97" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E97" s="3" t="n"/>
       <c r="F97" s="3" t="n"/>
-      <c r="G97" s="3" t="n"/>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Diabetes_mellitus_type_II</t>
+          <t>codetrt</t>
         </is>
       </c>
       <c r="B98" s="3" t="n"/>
@@ -2368,11 +2510,12 @@
       </c>
       <c r="F98" s="3" t="n"/>
       <c r="G98" s="3" t="n"/>
+      <c r="H98" s="3" t="n"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Creatinine</t>
+          <t>Serum_Glucose</t>
         </is>
       </c>
       <c r="B99" s="3" t="n"/>
@@ -2385,45 +2528,48 @@
       </c>
       <c r="F99" s="3" t="n"/>
       <c r="G99" s="3" t="n"/>
+      <c r="H99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Corsi_forw</t>
+          <t>NIHSS_5B</t>
         </is>
       </c>
       <c r="B100" s="3" t="n"/>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C100" s="3" t="n"/>
       <c r="D100" s="3" t="n"/>
       <c r="E100" s="3" t="n"/>
       <c r="F100" s="3" t="n"/>
       <c r="G100" s="3" t="n"/>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Corsi_back</t>
+          <t>NIHSS_6b_3m</t>
         </is>
       </c>
       <c r="B101" s="3" t="n"/>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C101" s="3" t="n"/>
       <c r="D101" s="3" t="n"/>
-      <c r="E101" s="3" t="n"/>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F101" s="3" t="n"/>
       <c r="G101" s="3" t="n"/>
+      <c r="H101" s="3" t="n"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Coagulation_disorder</t>
+          <t>EQ5D</t>
         </is>
       </c>
       <c r="B102" s="3" t="n"/>
@@ -2436,11 +2582,12 @@
       </c>
       <c r="F102" s="3" t="n"/>
       <c r="G102" s="3" t="n"/>
+      <c r="H102" s="3" t="n"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Clock</t>
+          <t>Barthel</t>
         </is>
       </c>
       <c r="B103" s="3" t="n"/>
@@ -2453,28 +2600,30 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H103" s="3" t="n"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Barthel</t>
+          <t>Clock</t>
         </is>
       </c>
       <c r="B104" s="3" t="n"/>
       <c r="C104" s="3" t="n"/>
       <c r="D104" s="3" t="n"/>
       <c r="E104" s="3" t="n"/>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F104" s="3" t="n"/>
       <c r="G104" s="3" t="n"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>BDI</t>
+          <t>Coagulation_disorder</t>
         </is>
       </c>
       <c r="B105" s="3" t="n"/>
@@ -2487,45 +2636,48 @@
       </c>
       <c r="F105" s="3" t="n"/>
       <c r="G105" s="3" t="n"/>
+      <c r="H105" s="3" t="n"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>HPT9_right</t>
+          <t>Corsi_back</t>
         </is>
       </c>
       <c r="B106" s="3" t="n"/>
-      <c r="C106" s="3" t="n"/>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D106" s="3" t="n"/>
       <c r="E106" s="3" t="n"/>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F106" s="3" t="n"/>
       <c r="G106" s="3" t="n"/>
+      <c r="H106" s="3" t="n"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Atrial_fibrillation</t>
+          <t>Corsi_forw</t>
         </is>
       </c>
       <c r="B107" s="3" t="n"/>
-      <c r="C107" s="3" t="n"/>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D107" s="3" t="n"/>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E107" s="3" t="n"/>
       <c r="F107" s="3" t="n"/>
       <c r="G107" s="3" t="n"/>
+      <c r="H107" s="3" t="n"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Arterial_hypertension</t>
+          <t>Creatinine</t>
         </is>
       </c>
       <c r="B108" s="3" t="n"/>
@@ -2538,11 +2690,12 @@
       </c>
       <c r="F108" s="3" t="n"/>
       <c r="G108" s="3" t="n"/>
+      <c r="H108" s="3" t="n"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Antihypertensives_drug</t>
+          <t>Diabetes_mellitus_type_II</t>
         </is>
       </c>
       <c r="B109" s="3" t="n"/>
@@ -2555,11 +2708,12 @@
       </c>
       <c r="F109" s="3" t="n"/>
       <c r="G109" s="3" t="n"/>
+      <c r="H109" s="3" t="n"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Antihypertensives</t>
+          <t>EQ5D_3m</t>
         </is>
       </c>
       <c r="B110" s="3" t="n"/>
@@ -2572,11 +2726,12 @@
       </c>
       <c r="F110" s="3" t="n"/>
       <c r="G110" s="3" t="n"/>
+      <c r="H110" s="3" t="n"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Antidiabetics_drug</t>
+          <t>NIHSS_6a_3m</t>
         </is>
       </c>
       <c r="B111" s="3" t="n"/>
@@ -2589,11 +2744,12 @@
       </c>
       <c r="F111" s="3" t="n"/>
       <c r="G111" s="3" t="n"/>
+      <c r="H111" s="3" t="n"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Antidiabetics</t>
+          <t>FHS</t>
         </is>
       </c>
       <c r="B112" s="3" t="n"/>
@@ -2606,11 +2762,12 @@
       </c>
       <c r="F112" s="3" t="n"/>
       <c r="G112" s="3" t="n"/>
+      <c r="H112" s="3" t="n"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Anticoagulants</t>
+          <t>FHS_3m</t>
         </is>
       </c>
       <c r="B113" s="3" t="n"/>
@@ -2623,45 +2780,48 @@
       </c>
       <c r="F113" s="3" t="n"/>
       <c r="G113" s="3" t="n"/>
+      <c r="H113" s="3" t="n"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ARAT_R</t>
+          <t>FMA</t>
         </is>
       </c>
       <c r="B114" s="3" t="n"/>
       <c r="C114" s="3" t="n"/>
       <c r="D114" s="3" t="n"/>
       <c r="E114" s="3" t="n"/>
-      <c r="F114" s="3" t="n"/>
-      <c r="G114" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="n"/>
+      <c r="H114" s="3" t="n"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ARAT_L</t>
+          <t>FMA_12m</t>
         </is>
       </c>
       <c r="B115" s="3" t="n"/>
       <c r="C115" s="3" t="n"/>
       <c r="D115" s="3" t="n"/>
       <c r="E115" s="3" t="n"/>
-      <c r="F115" s="3" t="n"/>
-      <c r="G115" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="n"/>
+      <c r="H115" s="3" t="n"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>AAT_sp</t>
+          <t>FMA_1m</t>
         </is>
       </c>
       <c r="B116" s="3" t="n"/>
@@ -2674,11 +2834,12 @@
         </is>
       </c>
       <c r="G116" s="3" t="n"/>
+      <c r="H116" s="3" t="n"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>AAT_re</t>
+          <t>FMA_3m</t>
         </is>
       </c>
       <c r="B117" s="3" t="n"/>
@@ -2691,45 +2852,48 @@
         </is>
       </c>
       <c r="G117" s="3" t="n"/>
+      <c r="H117" s="3" t="n"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>AAT_na</t>
+          <t>Fluency_phonemic</t>
         </is>
       </c>
       <c r="B118" s="3" t="n"/>
-      <c r="C118" s="3" t="n"/>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D118" s="3" t="n"/>
       <c r="E118" s="3" t="n"/>
-      <c r="F118" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F118" s="3" t="n"/>
       <c r="G118" s="3" t="n"/>
+      <c r="H118" s="3" t="n"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>AAT_co</t>
+          <t>BDI_3m</t>
         </is>
       </c>
       <c r="B119" s="3" t="n"/>
       <c r="C119" s="3" t="n"/>
       <c r="D119" s="3" t="n"/>
-      <c r="E119" s="3" t="n"/>
-      <c r="F119" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="n"/>
       <c r="G119" s="3" t="n"/>
+      <c r="H119" s="3" t="n"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>&lt;gene nomenclature&gt;</t>
+          <t>BDI</t>
         </is>
       </c>
       <c r="B120" s="3" t="n"/>
@@ -2742,28 +2906,30 @@
       </c>
       <c r="F120" s="3" t="n"/>
       <c r="G120" s="3" t="n"/>
+      <c r="H120" s="3" t="n"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>HPT9_left</t>
+          <t>Atrial_fibrillation</t>
         </is>
       </c>
       <c r="B121" s="3" t="n"/>
       <c r="C121" s="3" t="n"/>
       <c r="D121" s="3" t="n"/>
-      <c r="E121" s="3" t="n"/>
-      <c r="F121" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="n"/>
       <c r="G121" s="3" t="n"/>
+      <c r="H121" s="3" t="n"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Hb</t>
+          <t>Arterial_hypertension</t>
         </is>
       </c>
       <c r="B122" s="3" t="n"/>
@@ -2776,79 +2942,84 @@
       </c>
       <c r="F122" s="3" t="n"/>
       <c r="G122" s="3" t="n"/>
+      <c r="H122" s="3" t="n"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>NIHSS_6A</t>
+          <t>9HPT_ratio</t>
         </is>
       </c>
       <c r="B123" s="3" t="n"/>
       <c r="C123" s="3" t="n"/>
       <c r="D123" s="3" t="n"/>
       <c r="E123" s="3" t="n"/>
-      <c r="F123" s="3" t="n"/>
-      <c r="G123" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="n"/>
+      <c r="H123" s="3" t="n"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>NIHSS_11_3m</t>
+          <t>9HPT_ratio_12m</t>
         </is>
       </c>
       <c r="B124" s="3" t="n"/>
       <c r="C124" s="3" t="n"/>
       <c r="D124" s="3" t="n"/>
-      <c r="E124" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F124" s="3" t="n"/>
+      <c r="E124" s="3" t="n"/>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G124" s="3" t="n"/>
+      <c r="H124" s="3" t="n"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>NIHSS_5b_3m</t>
+          <t>9HPT_ratio_1m</t>
         </is>
       </c>
       <c r="B125" s="3" t="n"/>
       <c r="C125" s="3" t="n"/>
       <c r="D125" s="3" t="n"/>
-      <c r="E125" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F125" s="3" t="n"/>
+      <c r="E125" s="3" t="n"/>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G125" s="3" t="n"/>
+      <c r="H125" s="3" t="n"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>NIHSS_5a_3m</t>
+          <t>9HPT_ratio_3m</t>
         </is>
       </c>
       <c r="B126" s="3" t="n"/>
       <c r="C126" s="3" t="n"/>
       <c r="D126" s="3" t="n"/>
-      <c r="E126" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F126" s="3" t="n"/>
+      <c r="E126" s="3" t="n"/>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G126" s="3" t="n"/>
+      <c r="H126" s="3" t="n"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>NIHSS_5B</t>
+          <t>AAT_co</t>
         </is>
       </c>
       <c r="B127" s="3" t="n"/>
@@ -2861,11 +3032,12 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H127" s="3" t="n"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>9HPT_R</t>
+          <t>AAT_na</t>
         </is>
       </c>
       <c r="B128" s="3" t="n"/>
@@ -2878,113 +3050,120 @@
           <t>X</t>
         </is>
       </c>
+      <c r="H128" s="3" t="n"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>NIHSS_4_3m</t>
+          <t>AAT_re</t>
         </is>
       </c>
       <c r="B129" s="3" t="n"/>
       <c r="C129" s="3" t="n"/>
       <c r="D129" s="3" t="n"/>
-      <c r="E129" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E129" s="3" t="n"/>
       <c r="F129" s="3" t="n"/>
-      <c r="G129" s="3" t="n"/>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H129" s="3" t="n"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>NIHSS_3_3m</t>
+          <t>AAT_sp</t>
         </is>
       </c>
       <c r="B130" s="3" t="n"/>
       <c r="C130" s="3" t="n"/>
       <c r="D130" s="3" t="n"/>
-      <c r="E130" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E130" s="3" t="n"/>
       <c r="F130" s="3" t="n"/>
-      <c r="G130" s="3" t="n"/>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H130" s="3" t="n"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>NIHSS_2_3m</t>
+          <t>ARAT_L</t>
         </is>
       </c>
       <c r="B131" s="3" t="n"/>
       <c r="C131" s="3" t="n"/>
       <c r="D131" s="3" t="n"/>
-      <c r="E131" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E131" s="3" t="n"/>
       <c r="F131" s="3" t="n"/>
       <c r="G131" s="3" t="n"/>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>NIHSS_1c</t>
+          <t>ARAT_R</t>
         </is>
       </c>
       <c r="B132" s="3" t="n"/>
       <c r="C132" s="3" t="n"/>
       <c r="D132" s="3" t="n"/>
       <c r="E132" s="3" t="n"/>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F132" s="3" t="n"/>
       <c r="G132" s="3" t="n"/>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>NIHSS_1b</t>
+          <t>Anticoagulants</t>
         </is>
       </c>
       <c r="B133" s="3" t="n"/>
       <c r="C133" s="3" t="n"/>
       <c r="D133" s="3" t="n"/>
-      <c r="E133" s="3" t="n"/>
-      <c r="F133" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="n"/>
       <c r="G133" s="3" t="n"/>
+      <c r="H133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>NIHSS_1a</t>
+          <t>Antidiabetics</t>
         </is>
       </c>
       <c r="B134" s="3" t="n"/>
       <c r="C134" s="3" t="n"/>
       <c r="D134" s="3" t="n"/>
-      <c r="E134" s="3" t="n"/>
-      <c r="F134" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="n"/>
       <c r="G134" s="3" t="n"/>
+      <c r="H134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>NIHSS_1C_3m</t>
+          <t>Antidiabetics_drug</t>
         </is>
       </c>
       <c r="B135" s="3" t="n"/>
@@ -2997,11 +3176,12 @@
       </c>
       <c r="F135" s="3" t="n"/>
       <c r="G135" s="3" t="n"/>
+      <c r="H135" s="3" t="n"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>NIHSS_1B_3m</t>
+          <t>Antihypertensives</t>
         </is>
       </c>
       <c r="B136" s="3" t="n"/>
@@ -3014,11 +3194,12 @@
       </c>
       <c r="F136" s="3" t="n"/>
       <c r="G136" s="3" t="n"/>
+      <c r="H136" s="3" t="n"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>NIHSS_1A_3m</t>
+          <t>Antihypertensives_drug</t>
         </is>
       </c>
       <c r="B137" s="3" t="n"/>
@@ -3031,28 +3212,30 @@
       </c>
       <c r="F137" s="3" t="n"/>
       <c r="G137" s="3" t="n"/>
+      <c r="H137" s="3" t="n"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>NIHSS_12m</t>
+          <t>GDS_15</t>
         </is>
       </c>
       <c r="B138" s="3" t="n"/>
-      <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="C138" s="3" t="n"/>
       <c r="D138" s="3" t="n"/>
       <c r="E138" s="3" t="n"/>
       <c r="F138" s="3" t="n"/>
       <c r="G138" s="3" t="n"/>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>NIHSS_10_3m</t>
+          <t>Gastro_intestinal_bleeding</t>
         </is>
       </c>
       <c r="B139" s="3" t="n"/>
@@ -3065,130 +3248,138 @@
       </c>
       <c r="F139" s="3" t="n"/>
       <c r="G139" s="3" t="n"/>
+      <c r="H139" s="3" t="n"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Hct</t>
+          <t>HPT9_left</t>
         </is>
       </c>
       <c r="B140" s="3" t="n"/>
       <c r="C140" s="3" t="n"/>
       <c r="D140" s="3" t="n"/>
-      <c r="E140" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E140" s="3" t="n"/>
       <c r="F140" s="3" t="n"/>
-      <c r="G140" s="3" t="n"/>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H140" s="3" t="n"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>MOCA_visuospatial</t>
+          <t>NIHSS_11_3m</t>
         </is>
       </c>
       <c r="B141" s="3" t="n"/>
       <c r="C141" s="3" t="n"/>
       <c r="D141" s="3" t="n"/>
-      <c r="E141" s="3" t="n"/>
-      <c r="F141" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="n"/>
       <c r="G141" s="3" t="n"/>
+      <c r="H141" s="3" t="n"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>MOCA_total</t>
+          <t>NIHSS_1B_3m</t>
         </is>
       </c>
       <c r="B142" s="3" t="n"/>
       <c r="C142" s="3" t="n"/>
       <c r="D142" s="3" t="n"/>
-      <c r="E142" s="3" t="n"/>
-      <c r="F142" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="n"/>
       <c r="G142" s="3" t="n"/>
+      <c r="H142" s="3" t="n"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>MOCA_recall</t>
+          <t>NIHSS_1C_3m</t>
         </is>
       </c>
       <c r="B143" s="3" t="n"/>
       <c r="C143" s="3" t="n"/>
       <c r="D143" s="3" t="n"/>
-      <c r="E143" s="3" t="n"/>
-      <c r="F143" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="n"/>
       <c r="G143" s="3" t="n"/>
+      <c r="H143" s="3" t="n"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>MOCA_orientation</t>
+          <t>NIHSS_1a</t>
         </is>
       </c>
       <c r="B144" s="3" t="n"/>
       <c r="C144" s="3" t="n"/>
       <c r="D144" s="3" t="n"/>
       <c r="E144" s="3" t="n"/>
-      <c r="F144" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G144" s="3" t="n"/>
+      <c r="F144" s="3" t="n"/>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H144" s="3" t="n"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>MOCA_naming</t>
+          <t>NIHSS_1b</t>
         </is>
       </c>
       <c r="B145" s="3" t="n"/>
       <c r="C145" s="3" t="n"/>
       <c r="D145" s="3" t="n"/>
       <c r="E145" s="3" t="n"/>
-      <c r="F145" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G145" s="3" t="n"/>
+      <c r="F145" s="3" t="n"/>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H145" s="3" t="n"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>MOCA_language</t>
+          <t>NIHSS_1c</t>
         </is>
       </c>
       <c r="B146" s="3" t="n"/>
       <c r="C146" s="3" t="n"/>
       <c r="D146" s="3" t="n"/>
       <c r="E146" s="3" t="n"/>
-      <c r="F146" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G146" s="3" t="n"/>
+      <c r="F146" s="3" t="n"/>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H146" s="3" t="n"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>MOCA_attention</t>
+          <t>NIHSS_1m</t>
         </is>
       </c>
       <c r="B147" s="3" t="n"/>
@@ -3201,28 +3392,30 @@
         </is>
       </c>
       <c r="G147" s="3" t="n"/>
+      <c r="H147" s="3" t="n"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>MOCA_abstraction</t>
+          <t>NIHSS_2_3m</t>
         </is>
       </c>
       <c r="B148" s="3" t="n"/>
       <c r="C148" s="3" t="n"/>
       <c r="D148" s="3" t="n"/>
-      <c r="E148" s="3" t="n"/>
-      <c r="F148" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="n"/>
       <c r="G148" s="3" t="n"/>
+      <c r="H148" s="3" t="n"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>LMWH</t>
+          <t>NIHSS_3_3m</t>
         </is>
       </c>
       <c r="B149" s="3" t="n"/>
@@ -3235,11 +3428,12 @@
       </c>
       <c r="F149" s="3" t="n"/>
       <c r="G149" s="3" t="n"/>
+      <c r="H149" s="3" t="n"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Ischemic_stroke</t>
+          <t>NIHSS_4_3m</t>
         </is>
       </c>
       <c r="B150" s="3" t="n"/>
@@ -3252,45 +3446,48 @@
       </c>
       <c r="F150" s="3" t="n"/>
       <c r="G150" s="3" t="n"/>
+      <c r="H150" s="3" t="n"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Intracranial_haemorrhage</t>
+          <t>NIHSS_5A</t>
         </is>
       </c>
       <c r="B151" s="3" t="n"/>
       <c r="C151" s="3" t="n"/>
       <c r="D151" s="3" t="n"/>
-      <c r="E151" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E151" s="3" t="n"/>
       <c r="F151" s="3" t="n"/>
       <c r="G151" s="3" t="n"/>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>9HPT_R</t>
         </is>
       </c>
       <c r="B152" s="3" t="n"/>
       <c r="C152" s="3" t="n"/>
       <c r="D152" s="3" t="n"/>
-      <c r="E152" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="E152" s="3" t="n"/>
       <c r="F152" s="3" t="n"/>
       <c r="G152" s="3" t="n"/>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Hypercholesterolemia</t>
+          <t>NIHSS_5a_3m</t>
         </is>
       </c>
       <c r="B153" s="3" t="n"/>
@@ -3303,11 +3500,12 @@
       </c>
       <c r="F153" s="3" t="n"/>
       <c r="G153" s="3" t="n"/>
+      <c r="H153" s="3" t="n"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Heparine</t>
+          <t>NIHSS_5b_3m</t>
         </is>
       </c>
       <c r="B154" s="3" t="n"/>
@@ -3320,23 +3518,403 @@
       </c>
       <c r="F154" s="3" t="n"/>
       <c r="G154" s="3" t="n"/>
+      <c r="H154" s="3" t="n"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>time_follow_up_(days)</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>NIHSS_6A</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="n"/>
       <c r="C155" s="3" t="n"/>
       <c r="D155" s="3" t="n"/>
       <c r="E155" s="3" t="n"/>
       <c r="F155" s="3" t="n"/>
       <c r="G155" s="3" t="n"/>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>NIHSS_6B</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="n"/>
+      <c r="C156" s="3" t="n"/>
+      <c r="D156" s="3" t="n"/>
+      <c r="E156" s="3" t="n"/>
+      <c r="F156" s="3" t="n"/>
+      <c r="G156" s="3" t="n"/>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>NIHSS_1A_3m</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="n"/>
+      <c r="C157" s="3" t="n"/>
+      <c r="D157" s="3" t="n"/>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="n"/>
+      <c r="G157" s="3" t="n"/>
+      <c r="H157" s="3" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>NIHSS_10_3m</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="n"/>
+      <c r="C158" s="3" t="n"/>
+      <c r="D158" s="3" t="n"/>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="n"/>
+      <c r="G158" s="3" t="n"/>
+      <c r="H158" s="3" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>HPT9_right</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="n"/>
+      <c r="C159" s="3" t="n"/>
+      <c r="D159" s="3" t="n"/>
+      <c r="E159" s="3" t="n"/>
+      <c r="F159" s="3" t="n"/>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>MOCA_visuospatial</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="n"/>
+      <c r="C160" s="3" t="n"/>
+      <c r="D160" s="3" t="n"/>
+      <c r="E160" s="3" t="n"/>
+      <c r="F160" s="3" t="n"/>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H160" s="3" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Hb</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="n"/>
+      <c r="C161" s="3" t="n"/>
+      <c r="D161" s="3" t="n"/>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="n"/>
+      <c r="G161" s="3" t="n"/>
+      <c r="H161" s="3" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Hct</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="n"/>
+      <c r="C162" s="3" t="n"/>
+      <c r="D162" s="3" t="n"/>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F162" s="3" t="n"/>
+      <c r="G162" s="3" t="n"/>
+      <c r="H162" s="3" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Heparine</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="n"/>
+      <c r="C163" s="3" t="n"/>
+      <c r="D163" s="3" t="n"/>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="n"/>
+      <c r="G163" s="3" t="n"/>
+      <c r="H163" s="3" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Hypercholesterolemia</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="n"/>
+      <c r="C164" s="3" t="n"/>
+      <c r="D164" s="3" t="n"/>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="n"/>
+      <c r="G164" s="3" t="n"/>
+      <c r="H164" s="3" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="n"/>
+      <c r="C165" s="3" t="n"/>
+      <c r="D165" s="3" t="n"/>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="n"/>
+      <c r="G165" s="3" t="n"/>
+      <c r="H165" s="3" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Intracranial_haemorrhage</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="n"/>
+      <c r="C166" s="3" t="n"/>
+      <c r="D166" s="3" t="n"/>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F166" s="3" t="n"/>
+      <c r="G166" s="3" t="n"/>
+      <c r="H166" s="3" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Ischemic_stroke</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="n"/>
+      <c r="C167" s="3" t="n"/>
+      <c r="D167" s="3" t="n"/>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="n"/>
+      <c r="G167" s="3" t="n"/>
+      <c r="H167" s="3" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>LMWH</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="n"/>
+      <c r="C168" s="3" t="n"/>
+      <c r="D168" s="3" t="n"/>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F168" s="3" t="n"/>
+      <c r="G168" s="3" t="n"/>
+      <c r="H168" s="3" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>MOCA_abstraction</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="n"/>
+      <c r="C169" s="3" t="n"/>
+      <c r="D169" s="3" t="n"/>
+      <c r="E169" s="3" t="n"/>
+      <c r="F169" s="3" t="n"/>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H169" s="3" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>MOCA_attention</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="n"/>
+      <c r="C170" s="3" t="n"/>
+      <c r="D170" s="3" t="n"/>
+      <c r="E170" s="3" t="n"/>
+      <c r="F170" s="3" t="n"/>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H170" s="3" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>MOCA_language</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="n"/>
+      <c r="C171" s="3" t="n"/>
+      <c r="D171" s="3" t="n"/>
+      <c r="E171" s="3" t="n"/>
+      <c r="F171" s="3" t="n"/>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H171" s="3" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>MOCA_naming</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="n"/>
+      <c r="C172" s="3" t="n"/>
+      <c r="D172" s="3" t="n"/>
+      <c r="E172" s="3" t="n"/>
+      <c r="F172" s="3" t="n"/>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H172" s="3" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>MOCA_orientation</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="n"/>
+      <c r="C173" s="3" t="n"/>
+      <c r="D173" s="3" t="n"/>
+      <c r="E173" s="3" t="n"/>
+      <c r="F173" s="3" t="n"/>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H173" s="3" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>MOCA_recall</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="n"/>
+      <c r="C174" s="3" t="n"/>
+      <c r="D174" s="3" t="n"/>
+      <c r="E174" s="3" t="n"/>
+      <c r="F174" s="3" t="n"/>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H174" s="3" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>MOCA_total</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="n"/>
+      <c r="C175" s="3" t="n"/>
+      <c r="D175" s="3" t="n"/>
+      <c r="E175" s="3" t="n"/>
+      <c r="F175" s="3" t="n"/>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H175" s="3" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>time_follow_up_(days)</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="n"/>
+      <c r="D176" s="3" t="n"/>
+      <c r="E176" s="3" t="n"/>
+      <c r="F176" s="3" t="n"/>
+      <c r="G176" s="3" t="n"/>
+      <c r="H176" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>